<commit_message>
Collating TMP Porewater Data for ESS-DIVE
</commit_message>
<xml_diff>
--- a/processing_scripts/TEMPEST Event Timepoints.xlsx
+++ b/processing_scripts/TEMPEST Event Timepoints.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sinet-my.sharepoint.com/personal/readz_si_edu1/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://sinet-my.sharepoint.com/personal/readz_si_edu1/Documents/TEMPEST_Porewater/processing_scripts/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="88" documentId="8_{CA9949DD-0F11-4A90-B61A-C5ABCA71829E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{180A49BC-0EEE-4848-9326-38AC47DAC430}"/>
+  <xr:revisionPtr revIDLastSave="90" documentId="8_{CA9949DD-0F11-4A90-B61A-C5ABCA71829E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{471BB1EF-0ADB-4AC3-8B7E-FBE22AD925EB}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{0C84C050-F263-4047-B3A6-8DBB1A7831CA}"/>
+    <workbookView xWindow="-19320" yWindow="690" windowWidth="19440" windowHeight="14880" xr2:uid="{0C84C050-F263-4047-B3A6-8DBB1A7831CA}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -207,12 +207,18 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -227,9 +233,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="49" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -245,6 +252,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -673,58 +684,58 @@
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C8" s="1">
+      <c r="C8" s="2">
         <v>20230606</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C9" s="1">
+      <c r="C9" s="2">
         <v>20230607</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="2" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B10" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="1" t="s">
+      <c r="B10" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="1" t="s">
+      <c r="D10" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="1" t="s">
+      <c r="B11" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="D11" s="2" t="s">
         <v>21</v>
       </c>
     </row>
@@ -841,198 +852,198 @@
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A20" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B20" s="1" t="s">
+      <c r="A20" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C20" s="1">
+      <c r="C20" s="2">
         <v>20260608</v>
       </c>
-      <c r="D20" s="1" t="s">
+      <c r="D20" s="2" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A21" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B21" s="1" t="s">
+      <c r="A21" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C21" s="1">
+      <c r="C21" s="2">
         <v>20260609</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A22" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B22" s="1" t="s">
+      <c r="A22" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B22" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C22" s="1">
+      <c r="C22" s="2">
         <v>20260610</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A23" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B23" s="1" t="s">
+      <c r="A23" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C23" s="1">
+      <c r="C23" s="2">
         <v>20260611</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="2" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A24" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B24" s="1" t="s">
+      <c r="A24" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B24" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C24" s="1">
+      <c r="C24" s="2">
         <v>20260608</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="2" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A25" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B25" s="1" t="s">
+      <c r="A25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C25" s="1">
+      <c r="C25" s="2">
         <v>20260609</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A26" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B26" s="1" t="s">
+      <c r="A26" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B26" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C26" s="1">
+      <c r="C26" s="2">
         <v>20260610</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A27" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B27" s="1" t="s">
+      <c r="A27" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B27" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C27" s="1">
+      <c r="C27" s="2">
         <v>20260611</v>
       </c>
-      <c r="D27" s="1" t="s">
+      <c r="D27" s="2" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A28" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C28" s="1" t="s">
+      <c r="A28" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="D28" s="1" t="s">
+      <c r="D28" s="2" t="s">
         <v>46</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A29" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C29" s="1" t="s">
+      <c r="A29" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="2" t="s">
         <v>47</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A30" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C30" s="1" t="s">
+      <c r="A30" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="D30" s="1" t="s">
+      <c r="D30" s="2" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A31" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C31" s="1" t="s">
+      <c r="A31" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D31" s="1" t="s">
+      <c r="D31" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A32" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C32" s="1" t="s">
+      <c r="A32" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="D32" s="1" t="s">
+      <c r="D32" s="2" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C33" s="1" t="s">
+      <c r="A33" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D33" s="1" t="s">
+      <c r="D33" s="2" t="s">
         <v>48</v>
       </c>
     </row>

</xml_diff>